<commit_message>
fix: resolve broken and not-found external links across Scopus, Clarivate, and homepages
</commit_message>
<xml_diff>
--- a/faculty_publications_output.xlsx
+++ b/faculty_publications_output.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,11 +52,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="006C757D"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00084298"/>
       <sz val="10"/>
@@ -68,7 +63,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -97,12 +92,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
         <bgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E9ECEF"/>
-        <bgColor rgb="00E9ECEF"/>
       </patternFill>
     </fill>
     <fill>
@@ -144,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,22 +168,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -728,7 +702,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -763,7 +737,7 @@
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -791,9 +765,9 @@
           <t>409-440</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Journal Homepage</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -807,7 +781,7 @@
         </is>
       </c>
       <c r="S2" s="6" t="n">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="T2" s="6" t="n">
         <v>1</v>
@@ -822,9 +796,9 @@
           <t>Scopus Source Proof</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>SCImago SJR Proof</t>
         </is>
       </c>
       <c r="X2" s="3" t="inlineStr">
@@ -846,7 +820,7 @@
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -881,7 +855,7 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I3" s="9" t="inlineStr">
@@ -909,9 +883,9 @@
           <t>346-378</t>
         </is>
       </c>
-      <c r="P3" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Journal Homepage</t>
         </is>
       </c>
       <c r="Q3" s="7" t="inlineStr">
@@ -925,7 +899,7 @@
         </is>
       </c>
       <c r="S3" s="10" t="n">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="T3" s="10" t="n">
         <v>1</v>
@@ -940,9 +914,9 @@
           <t>Scopus Source Proof</t>
         </is>
       </c>
-      <c r="W3" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="W3" s="8" t="inlineStr">
+        <is>
+          <t>SCImago SJR Proof</t>
         </is>
       </c>
       <c r="X3" s="8" t="inlineStr">
@@ -964,7 +938,7 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1034,7 +1008,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
+          <t>Scopus Verified (Conference Paper)</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
@@ -1043,14 +1017,14 @@
         </is>
       </c>
       <c r="S4" s="6" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="T4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" s="3" t="inlineStr">
-        <is>
-          <t>Clarivate MJL Proof</t>
+        <v>1</v>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
@@ -1082,7 +1056,7 @@
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1102,22 +1076,22 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Direction Dependent Non-gaussianity in High-z Supernova Data</t>
+          <t>High-z Type Ia supernova data: non-Gaussianity and direction dependence</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Shashikant Gupta (Amity University Gurugram); Meghendra Singh</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Monthly Notices of the Royal Astronomical Society</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0035-8711</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
@@ -1130,91 +1104,85 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="K5" s="9" t="n">
+        <v>2014</v>
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>April</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>440</t>
         </is>
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O5" s="9" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P5" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>3257-3261</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Journal Homepage</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>No ISSN/ISBN Available</t>
-        </is>
-      </c>
-      <c r="R5" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S5" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T5" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U5" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V5" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W5" s="9" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X5" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y5" s="13" t="inlineStr">
-        <is>
-          <t>https://vidwan.inflibnet.ac.in/profile/419754</t>
+          <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S5" s="10" t="n">
+        <v>501</v>
+      </c>
+      <c r="T5" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="U5" s="8" t="inlineStr">
+        <is>
+          <t>Clarivate MJL Proof</t>
+        </is>
+      </c>
+      <c r="V5" s="8" t="inlineStr">
+        <is>
+          <t>Scopus Source Proof</t>
+        </is>
+      </c>
+      <c r="W5" s="8" t="inlineStr">
+        <is>
+          <t>SCImago SJR Proof</t>
+        </is>
+      </c>
+      <c r="X5" s="8" t="inlineStr">
+        <is>
+          <t>10.1093/mnras/stu416</t>
+        </is>
+      </c>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>10.1093/mnras/stu416</t>
         </is>
       </c>
       <c r="Z5" s="9" t="inlineStr">
         <is>
-          <t>DOI not available</t>
+          <t>Success</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1234,22 +1202,22 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Non-Gaussianity and direction dependent systematics in HST key project data</t>
+          <t>Non-Gaussianity and direction-dependent systematics in HST Key Project data</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Shashikant Gupta (Raman Research Institute, Indian Institute of Science Bangalore); Tarun Deep Saini (Indian Institute of Science Bangalore)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Monthly Notices of the Royal Astronomical Society</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0035-8711</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1262,91 +1230,85 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="K6" s="4" t="n">
+        <v>2011</v>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>July</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>415</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P6" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>2594-2599</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Journal Homepage</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>No ISSN/ISBN Available</t>
-        </is>
-      </c>
-      <c r="R6" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S6" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U6" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V6" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W6" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X6" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y6" s="15" t="inlineStr">
-        <is>
-          <t>https://vidwan.inflibnet.ac.in/profile/419754</t>
+          <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>501</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>Clarivate MJL Proof</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Scopus Source Proof</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="inlineStr">
+        <is>
+          <t>SCImago SJR Proof</t>
+        </is>
+      </c>
+      <c r="X6" s="3" t="inlineStr">
+        <is>
+          <t>10.1111/j.1365-2966.2011.18882.x</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>10.1111/j.1365-2966.2011.18882.x</t>
         </is>
       </c>
       <c r="Z6" s="4" t="inlineStr">
         <is>
-          <t>DOI not available</t>
+          <t>Success</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1433,7 +1395,7 @@
         </is>
       </c>
       <c r="S7" s="10" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="T7" s="10" t="n">
         <v>8</v>
@@ -1472,7 +1434,7 @@
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1492,22 +1454,22 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>High-z Supernova Type Ia Data: non-Gaussianity and Direction Dependence</t>
+          <t>High-z Type Ia supernova data: non-Gaussianity and direction dependence</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Shashikant Gupta (Amity University Gurugram); Meghendra Singh</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Monthly Notices of the Royal Astronomical Society</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0035-8711</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1520,91 +1482,85 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="K8" s="4" t="n">
+        <v>2014</v>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>April</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>440</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
+          <t>3257-3261</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Journal Homepage</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>No ISSN/ISBN Available</t>
-        </is>
-      </c>
-      <c r="R8" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S8" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U8" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V8" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X8" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y8" s="15" t="inlineStr">
-        <is>
-          <t>https://vidwan.inflibnet.ac.in/profile/419754</t>
+          <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>501</v>
+      </c>
+      <c r="T8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>Clarivate MJL Proof</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="inlineStr">
+        <is>
+          <t>Scopus Source Proof</t>
+        </is>
+      </c>
+      <c r="W8" s="3" t="inlineStr">
+        <is>
+          <t>SCImago SJR Proof</t>
+        </is>
+      </c>
+      <c r="X8" s="3" t="inlineStr">
+        <is>
+          <t>10.1093/mnras/stu416</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
+          <t>10.1093/mnras/stu416</t>
         </is>
       </c>
       <c r="Z8" s="4" t="inlineStr">
         <is>
-          <t>DOI not available</t>
+          <t>Success</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1685,13 +1641,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R9" s="16" t="inlineStr">
+      <c r="R9" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S9" s="10" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T9" s="10" t="n">
         <v>2</v>
@@ -1730,7 +1686,7 @@
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1817,7 +1773,7 @@
         </is>
       </c>
       <c r="S10" s="6" t="n">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="T10" s="6" t="n">
         <v>7</v>
@@ -1856,7 +1812,7 @@
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1937,13 +1893,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R11" s="16" t="inlineStr">
+      <c r="R11" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S11" s="10" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T11" s="10" t="n">
         <v>2</v>
@@ -1982,7 +1938,7 @@
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2063,7 +2019,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R12" s="16" t="inlineStr">
+      <c r="R12" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
@@ -2108,7 +2064,7 @@
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -2178,10 +2134,10 @@
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
-        </is>
-      </c>
-      <c r="R13" s="16" t="inlineStr">
+          <t>Scopus Verified (Book Chapter)</t>
+        </is>
+      </c>
+      <c r="R13" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
@@ -2192,9 +2148,9 @@
       <c r="T13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="U13" s="8" t="inlineStr">
-        <is>
-          <t>Clarivate MJL Proof</t>
+      <c r="U13" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
       <c r="V13" s="8" t="inlineStr">
@@ -2226,7 +2182,7 @@
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -2307,13 +2263,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R14" s="16" t="inlineStr">
+      <c r="R14" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S14" s="6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T14" s="6" t="n">
         <v>0</v>
@@ -2352,7 +2308,7 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -2433,7 +2389,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R15" s="17" t="inlineStr">
+      <c r="R15" s="12" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
@@ -2478,7 +2434,7 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -2559,7 +2515,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R16" s="17" t="inlineStr">
+      <c r="R16" s="12" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
@@ -2604,7 +2560,7 @@
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -2685,7 +2641,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R17" s="17" t="inlineStr">
+      <c r="R17" s="12" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
@@ -2730,7 +2686,7 @@
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -2811,7 +2767,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R18" s="17" t="inlineStr">
+      <c r="R18" s="12" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
@@ -2856,7 +2812,7 @@
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -2937,7 +2893,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R19" s="16" t="inlineStr">
+      <c r="R19" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
@@ -2982,7 +2938,7 @@
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -3063,13 +3019,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R20" s="16" t="inlineStr">
+      <c r="R20" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S20" s="6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T20" s="6" t="n">
         <v>6</v>
@@ -3108,7 +3064,7 @@
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -3191,7 +3147,7 @@
         </is>
       </c>
       <c r="S21" s="10" t="n">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="T21" s="10" t="n">
         <v>2</v>
@@ -3230,7 +3186,7 @@
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -3307,13 +3263,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R22" s="16" t="inlineStr">
+      <c r="R22" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S22" s="6" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="T22" s="6" t="n">
         <v>3</v>
@@ -3352,7 +3308,7 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -3429,13 +3385,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R23" s="16" t="inlineStr">
+      <c r="R23" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S23" s="10" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="T23" s="10" t="n">
         <v>9</v>
@@ -3474,7 +3430,7 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -3557,7 +3513,7 @@
         </is>
       </c>
       <c r="S24" s="6" t="n">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="T24" s="6" t="n">
         <v>10</v>
@@ -3596,7 +3552,7 @@
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -3677,13 +3633,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R25" s="16" t="inlineStr">
+      <c r="R25" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S25" s="10" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T25" s="10" t="n">
         <v>3</v>
@@ -3722,7 +3678,7 @@
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -3803,13 +3759,13 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R26" s="16" t="inlineStr">
+      <c r="R26" s="11" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
       </c>
       <c r="S26" s="6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="T26" s="6" t="n">
         <v>14</v>
@@ -3848,7 +3804,7 @@
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -3925,7 +3881,7 @@
           <t>Scopus Verified | SCI/SCIE (Verify on Clarivate MJL)</t>
         </is>
       </c>
-      <c r="R27" s="17" t="inlineStr">
+      <c r="R27" s="12" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
@@ -3970,7 +3926,7 @@
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -4057,10 +4013,10 @@
         </is>
       </c>
       <c r="S28" s="6" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="T28" s="6" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="U28" s="3" t="inlineStr">
         <is>
@@ -4096,7 +4052,7 @@
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -4183,7 +4139,7 @@
         </is>
       </c>
       <c r="S29" s="10" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="T29" s="10" t="n">
         <v>31</v>
@@ -4222,7 +4178,7 @@
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -4309,7 +4265,7 @@
         </is>
       </c>
       <c r="S30" s="6" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>3</v>
@@ -4348,7 +4304,7 @@
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Dr Shashikant Gupta</t>
+          <t>Dr. Shashikant Gupta</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -4471,167 +4427,181 @@
   <autoFilter ref="A1:Z31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V4" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y5" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y6" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V7" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y8" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V11" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V12" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U13" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V13" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V14" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W14" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V16" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W16" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W17" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W18" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W19" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W20" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V21" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W21" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V22" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W22" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V23" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W23" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V24" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W24" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V25" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W25" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V26" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W26" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V27" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W27" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V28" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W28" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V29" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W29" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V30" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W30" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W31" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X5" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W6" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X6" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U7" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V7" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W7" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X7" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U8" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V8" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W8" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X8" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U9" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V9" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W9" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X9" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U10" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V10" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W10" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U11" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V11" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W11" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X11" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U12" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V12" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W12" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X12" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V13" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W13" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X13" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U14" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V14" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W14" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X14" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U15" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V15" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W15" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X15" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U16" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V16" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W16" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X16" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P17" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U17" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V17" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W17" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X17" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P18" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U18" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V18" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W18" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X18" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U19" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V19" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W19" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X19" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U20" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V20" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W20" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X20" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P21" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U21" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V21" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W21" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X21" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U22" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V22" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W22" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X22" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U23" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V23" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W23" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U24" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V24" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W24" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U25" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V25" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W25" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U26" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V26" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W26" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U27" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V27" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W27" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U28" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V28" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W28" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X28" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P29" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U29" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V29" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W29" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X29" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P30" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U30" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V30" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W30" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X30" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P31" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="U31" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="V31" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="W31" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X31" r:id="rId176"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: ensure uniform cell formatting and clean defaults for missing bibliographic fields
</commit_message>
<xml_diff>
--- a/faculty_publications_output.xlsx
+++ b/faculty_publications_output.xlsx
@@ -758,8 +758,16 @@
           <t>June</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
           <t>409-440</t>
@@ -876,8 +884,16 @@
           <t>June</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr"/>
-      <c r="N3" s="9" t="inlineStr"/>
+      <c r="M3" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O3" s="9" t="inlineStr">
         <is>
           <t>346-378</t>
@@ -994,8 +1010,16 @@
           <t>January</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
           <t>79-88</t>
@@ -2120,8 +2144,16 @@
           <t>January</t>
         </is>
       </c>
-      <c r="M13" s="9" t="inlineStr"/>
-      <c r="N13" s="9" t="inlineStr"/>
+      <c r="M13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
           <t>397-401</t>
@@ -3125,7 +3157,11 @@
           <t>866</t>
         </is>
       </c>
-      <c r="N21" s="9" t="inlineStr"/>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
           <t>139500</t>
@@ -3247,7 +3283,11 @@
           <t>120</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
           <t>102411</t>
@@ -3369,7 +3409,11 @@
           <t>34</t>
         </is>
       </c>
-      <c r="N23" s="9" t="inlineStr"/>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
           <t>100894</t>
@@ -3491,7 +3535,11 @@
           <t>840</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
           <t>137886</t>
@@ -3870,7 +3918,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="O27" s="9" t="inlineStr"/>
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P27" s="8" t="inlineStr">
         <is>
           <t>Journal Homepage</t>
@@ -4370,7 +4422,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="O31" s="9" t="inlineStr"/>
+      <c r="O31" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
           <t>Journal Homepage</t>

</xml_diff>